<commit_message>
Scripts 07-16 completos: meta-análise, valor incremental, QC todas 4 coortes
- 07_survival_analysis_SCANB: fix time_col (os_time_months) + Cadj corrigido
  SCANB: HR=1.923, C-index=0.698 (0.668-0.729), N=3069
- 08_meta_survival: Meta HR=1.472 (1.21-1.80), I2=90.6%, 4 coortes
  fix geom_errorbarh → geom_errorbar(orientation='y')
- 11_incremental_value: fix ENDPOINT_MAP, fix coxph concordance, CORE-A NA filter
  ΔC: SCANB=+0.030, TCGA=+0.038, METABRIC=+0.142, GSE20685=+0.093
- 13_qc: correlações off-diagonal computadas
- 14_qc: PCA forense METABRIC, 1 outlier (MB-5135)
- 15_qc: 44 PASS, 0 FAIL (fix column names: os_time_months, dss_time_months)
- 16_qc: 8 PASS, 0 FAIL (reinstall lubridate)
- FigS5 METABRIC Sensitivity regenerada
- Novos artefatos: Fig3-5 (main), FigS3-4 (supp), calibração 60m, meta-análise LOO

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/results/main/Table3_Survival_Performance_ByCohort.xlsx
+++ b/results/main/Table3_Survival_Performance_ByCohort.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="29">
   <si>
     <t xml:space="preserve">Cohort</t>
   </si>
@@ -38,10 +38,10 @@
     <t xml:space="preserve">C_adj (95%CI)</t>
   </si>
   <si>
-    <t xml:space="preserve">HR multi (CORE-A)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">p (multi)</t>
+    <t xml:space="preserve">HR age-adj</t>
+  </si>
+  <si>
+    <t xml:space="preserve">p (age-adj)</t>
   </si>
   <si>
     <t xml:space="preserve">TCGA_BRCA</t>
@@ -59,7 +59,10 @@
     <t xml:space="preserve">0.624 (0.572–0.678)</t>
   </si>
   <si>
-    <t xml:space="preserve">—</t>
+    <t xml:space="preserve">1.27 (1.09–1.48)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.0023</t>
   </si>
   <si>
     <t xml:space="preserve">METABRIC</t>
@@ -77,6 +80,12 @@
     <t xml:space="preserve">0.638 (0.615–0.659)</t>
   </si>
   <si>
+    <t xml:space="preserve">1.41 (1.31–1.53)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3.07e-19</t>
+  </si>
+  <si>
     <t xml:space="preserve">GSE20685</t>
   </si>
   <si>
@@ -87,6 +96,9 @@
   </si>
   <si>
     <t xml:space="preserve">0.623 (0.562–0.683)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.0032</t>
   </si>
 </sst>
 </file>
@@ -472,8 +484,8 @@
     <col min="6" max="6" width="16.145" hidden="0" customWidth="1"/>
     <col min="7" max="7" width="7.71" hidden="0" customWidth="1"/>
     <col min="8" max="8" width="18.7175" hidden="0" customWidth="1"/>
-    <col min="9" max="9" width="17.71" hidden="0" customWidth="1"/>
-    <col min="10" max="10" width="9.71" hidden="0" customWidth="1"/>
+    <col min="9" max="9" width="16.145" hidden="0" customWidth="1"/>
+    <col min="10" max="10" width="11.71" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -537,15 +549,15 @@
         <v>15</v>
       </c>
       <c r="J2" s="2" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C3" s="3" t="n">
         <v>1978</v>
@@ -557,24 +569,24 @@
         <v>159</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="I3" s="3" t="s">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="J3" s="3" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>11</v>
@@ -589,19 +601,19 @@
         <v>112.8</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="J4" s="2" t="s">
-        <v>15</v>
+        <v>28</v>
       </c>
     </row>
   </sheetData>

</xml_diff>